<commit_message>
Regenerate the original example workbook with the new parity columns filled in
Same 20-organization dataset as before, re-ported from
Organization_Template_Alternate_example_data.xlsx now that Main Org
record and the Emails overflow sheet have somewhere to put every field
an instance-1 alias/address/phone/email can carry.

Re-ran process_template.php and diffed organizations.json,
contacts.json, interfaces.json, credentials.json, notes.json,
categories.json, organization_types.json, and note_types.json against
the alternate template's own run field-by-field: all eight match
exactly now, zero differences -- confirming the previous commit's new
columns actually close the gap, not just for this one field
combination but for the full dataset.
</commit_message>
<xml_diff>
--- a/Organization_Template_example_data.xlsx
+++ b/Organization_Template_example_data.xlsx
@@ -1797,7 +1797,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T28"/>
+  <dimension ref="A1:AD28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11.42578125" customWidth="1" style="23" min="1" max="1"/>
@@ -1851,85 +1851,135 @@
       </c>
       <c r="D5" s="32" t="inlineStr">
         <is>
+          <t>ALT NAME DESCRIPTION</t>
+        </is>
+      </c>
+      <c r="E5" s="32" t="inlineStr">
+        <is>
           <t>Vendor (Yes/No)</t>
         </is>
       </c>
-      <c r="E5" s="32" t="inlineStr">
+      <c r="F5" s="32" t="inlineStr">
         <is>
           <t>ORG status (Active/Inactive/Pending)*</t>
         </is>
       </c>
-      <c r="F5" s="32" t="inlineStr">
+      <c r="G5" s="32" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="G5" s="32" t="inlineStr">
+      <c r="H5" s="32" t="inlineStr">
         <is>
           <t xml:space="preserve">ADDR1 </t>
         </is>
       </c>
-      <c r="H5" s="32" t="inlineStr">
+      <c r="I5" s="32" t="inlineStr">
         <is>
           <t>ADDR2</t>
         </is>
       </c>
-      <c r="I5" s="32" t="inlineStr">
+      <c r="J5" s="32" t="inlineStr">
         <is>
           <t>CITY</t>
         </is>
       </c>
-      <c r="J5" s="32" t="inlineStr">
+      <c r="K5" s="32" t="inlineStr">
         <is>
           <t>REGION</t>
         </is>
       </c>
-      <c r="K5" s="32" t="inlineStr">
+      <c r="L5" s="32" t="inlineStr">
         <is>
           <t>POSTAL CODE</t>
         </is>
       </c>
-      <c r="L5" s="32" t="inlineStr">
+      <c r="M5" s="32" t="inlineStr">
         <is>
           <t>COUNTRY</t>
         </is>
       </c>
-      <c r="M5" s="32" t="inlineStr">
+      <c r="N5" s="32" t="inlineStr">
+        <is>
+          <t>ADDR LANGUAGE</t>
+        </is>
+      </c>
+      <c r="O5" s="32" t="inlineStr">
+        <is>
+          <t>ADDR CATEGORIES</t>
+        </is>
+      </c>
+      <c r="P5" s="32" t="inlineStr">
         <is>
           <t>PHONE</t>
         </is>
       </c>
-      <c r="N5" s="32" t="inlineStr">
+      <c r="Q5" s="32" t="inlineStr">
+        <is>
+          <t>PHONE TYPE</t>
+        </is>
+      </c>
+      <c r="R5" s="32" t="inlineStr">
+        <is>
+          <t>PHONE LANGUAGE</t>
+        </is>
+      </c>
+      <c r="S5" s="32" t="inlineStr">
+        <is>
+          <t>PHONE CATEGORIES</t>
+        </is>
+      </c>
+      <c r="T5" s="32" t="inlineStr">
         <is>
           <t>FAX</t>
         </is>
       </c>
-      <c r="O5" s="32" t="inlineStr">
+      <c r="U5" s="32" t="inlineStr">
         <is>
           <t>EMAIL</t>
         </is>
       </c>
-      <c r="P5" s="32" t="inlineStr">
+      <c r="V5" s="32" t="inlineStr">
+        <is>
+          <t>EMAIL DESCRIPTION</t>
+        </is>
+      </c>
+      <c r="W5" s="32" t="inlineStr">
+        <is>
+          <t>EMAIL LANGUAGE</t>
+        </is>
+      </c>
+      <c r="X5" s="32" t="inlineStr">
+        <is>
+          <t>EMAIL CATEGORIES</t>
+        </is>
+      </c>
+      <c r="Y5" s="32" t="inlineStr">
         <is>
           <t>URL</t>
         </is>
       </c>
-      <c r="Q5" s="31" t="inlineStr">
+      <c r="Z5" s="31" t="inlineStr">
         <is>
           <t>URL DESCRIPTION</t>
         </is>
       </c>
-      <c r="R5" s="31" t="inlineStr">
+      <c r="AA5" s="32" t="inlineStr">
+        <is>
+          <t>URL LANGUAGE</t>
+        </is>
+      </c>
+      <c r="AB5" s="31" t="inlineStr">
         <is>
           <t>URL NOTE</t>
         </is>
       </c>
-      <c r="S5" s="31" t="inlineStr">
+      <c r="AC5" s="31" t="inlineStr">
         <is>
           <t>URL CATEGORIES</t>
         </is>
       </c>
-      <c r="T5" s="31" t="inlineStr">
+      <c r="AD5" s="31" t="inlineStr">
         <is>
           <t>ORG TYPE</t>
         </is>
@@ -1951,83 +2001,118 @@
           <t>GT Solutions</t>
         </is>
       </c>
-      <c r="D6" s="25" t="inlineStr">
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Common shorthand used internally</t>
+        </is>
+      </c>
+      <c r="E6" s="25" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E6" s="25" t="inlineStr">
+      <c r="F6" s="25" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="F6" s="25" t="inlineStr">
+      <c r="G6" s="25" t="inlineStr">
         <is>
           <t>Full-service technology vendor with global reach.</t>
         </is>
       </c>
-      <c r="G6" s="25" t="inlineStr">
+      <c r="H6" s="25" t="inlineStr">
         <is>
           <t>100 Innovation Way</t>
         </is>
       </c>
-      <c r="H6" s="25" t="inlineStr">
+      <c r="I6" s="25" t="inlineStr">
         <is>
           <t>Suite 400</t>
         </is>
       </c>
-      <c r="I6" s="25" t="inlineStr">
+      <c r="J6" s="25" t="inlineStr">
         <is>
           <t>Austin</t>
         </is>
       </c>
-      <c r="J6" s="25" t="inlineStr">
+      <c r="K6" s="25" t="inlineStr">
         <is>
           <t>TX</t>
         </is>
       </c>
-      <c r="K6" s="25" t="inlineStr">
+      <c r="L6" s="25" t="inlineStr">
         <is>
           <t>73301</t>
         </is>
       </c>
-      <c r="L6" s="25" t="inlineStr">
+      <c r="M6" s="25" t="inlineStr">
         <is>
           <t>USA</t>
         </is>
       </c>
-      <c r="M6" s="25" t="inlineStr">
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>Billing;Shipping</t>
+        </is>
+      </c>
+      <c r="P6" s="25" t="inlineStr">
         <is>
           <t>512-555-0101</t>
         </is>
       </c>
-      <c r="N6" s="25" t="n"/>
-      <c r="O6" s="25" t="inlineStr">
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>Office</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>Sales;Support</t>
+        </is>
+      </c>
+      <c r="T6" s="25" t="n"/>
+      <c r="U6" s="25" t="inlineStr">
         <is>
           <t>info@globaltech.example</t>
         </is>
       </c>
-      <c r="P6" s="6" t="inlineStr">
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>General inquiries</t>
+        </is>
+      </c>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>eng</t>
+        </is>
+      </c>
+      <c r="X6" t="inlineStr">
+        <is>
+          <t>Support;Sales</t>
+        </is>
+      </c>
+      <c r="Y6" s="6" t="inlineStr">
         <is>
           <t>https://www.globaltech.example</t>
         </is>
       </c>
-      <c r="Q6" t="inlineStr">
+      <c r="Z6" t="inlineStr">
         <is>
           <t>Corporate site</t>
         </is>
       </c>
-      <c r="R6" t="inlineStr">
+      <c r="AB6" t="inlineStr">
         <is>
           <t>Primary marketing site</t>
         </is>
       </c>
-      <c r="S6" t="inlineStr">
+      <c r="AC6" t="inlineStr">
         <is>
           <t>Support</t>
         </is>
       </c>
-      <c r="T6" t="inlineStr">
+      <c r="AD6" t="inlineStr">
         <is>
           <t>Vendor|Publisher</t>
         </is>
@@ -2051,60 +2136,80 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
+          <t>Short form</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="G7" t="inlineStr">
         <is>
           <t>Regional book and media distributor.</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="H7" t="inlineStr">
         <is>
           <t>55 Prairie Ave</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="J7" t="inlineStr">
         <is>
           <t>Wichita</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="K7" t="inlineStr">
         <is>
           <t>KS</t>
         </is>
       </c>
-      <c r="K7" s="10" t="inlineStr">
+      <c r="L7" s="10" t="inlineStr">
         <is>
           <t>67202</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr">
+      <c r="M7" t="inlineStr">
         <is>
           <t>USA</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr">
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>Shipping</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
         <is>
           <t>316-555-0200</t>
         </is>
       </c>
-      <c r="O7" s="7" t="inlineStr">
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>Office</t>
+        </is>
+      </c>
+      <c r="U7" s="7" t="inlineStr">
         <is>
           <t>contact@prairiebooks.example</t>
         </is>
       </c>
-      <c r="P7" s="9" t="inlineStr">
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>eng</t>
+        </is>
+      </c>
+      <c r="Y7" s="9" t="inlineStr">
         <is>
           <t>https://www.prairiebooks.example</t>
         </is>
       </c>
-      <c r="T7" t="inlineStr">
+      <c r="AD7" t="inlineStr">
         <is>
           <t>Vendor</t>
         </is>
@@ -2126,62 +2231,87 @@
           <t>NorthStar</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="G8" t="inlineStr">
         <is>
           <t>Library automation and cataloging services.</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="H8" t="inlineStr">
         <is>
           <t>12 Polaris Blvd</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="J8" t="inlineStr">
         <is>
           <t>Minneapolis</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="K8" t="inlineStr">
         <is>
           <t>MN</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr">
+      <c r="L8" t="inlineStr">
         <is>
           <t>55401</t>
         </is>
       </c>
-      <c r="L8" t="inlineStr">
+      <c r="M8" t="inlineStr">
         <is>
           <t>USA</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr">
+      <c r="P8" t="inlineStr">
         <is>
           <t>612-555-0300</t>
         </is>
       </c>
-      <c r="O8" s="7" t="inlineStr">
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>Office</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>Support</t>
+        </is>
+      </c>
+      <c r="U8" s="7" t="inlineStr">
         <is>
           <t>help@northstarlib.example</t>
         </is>
       </c>
-      <c r="P8" t="inlineStr">
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>Support desk</t>
+        </is>
+      </c>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>eng</t>
+        </is>
+      </c>
+      <c r="X8" t="inlineStr">
+        <is>
+          <t>Support</t>
+        </is>
+      </c>
+      <c r="Y8" t="inlineStr">
         <is>
           <t>https://www.northstarlib.example</t>
         </is>
       </c>
-      <c r="T8" t="inlineStr">
+      <c r="AD8" t="inlineStr">
         <is>
           <t>Service Provider</t>
         </is>
@@ -2203,62 +2333,77 @@
           <t>Heritage Group</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="F9" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="G9" t="inlineStr">
         <is>
           <t>Archival preservation and conservation services.</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="H9" t="inlineStr">
         <is>
           <t>77 Archive Ln</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="J9" t="inlineStr">
         <is>
           <t>Boston</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr">
+      <c r="K9" t="inlineStr">
         <is>
           <t>MA</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr">
+      <c r="L9" t="inlineStr">
         <is>
           <t>02108</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr">
+      <c r="M9" t="inlineStr">
         <is>
           <t>USA</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr">
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>Shipping</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
         <is>
           <t>617-555-0400</t>
         </is>
       </c>
-      <c r="O9" s="7" t="inlineStr">
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>Office</t>
+        </is>
+      </c>
+      <c r="U9" s="7" t="inlineStr">
         <is>
           <t>info@heritagepres.example</t>
         </is>
       </c>
-      <c r="P9" s="7" t="inlineStr">
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>eng</t>
+        </is>
+      </c>
+      <c r="Y9" s="7" t="inlineStr">
         <is>
           <t>https://www.heritagepres.example</t>
         </is>
       </c>
-      <c r="T9" t="inlineStr">
+      <c r="AD9" t="inlineStr">
         <is>
           <t>Material Supplier</t>
         </is>
@@ -2280,67 +2425,97 @@
           <t>Summit Data</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="F10" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="G10" t="inlineStr">
         <is>
           <t>Data hosting and discovery platform provider.</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="H10" t="inlineStr">
         <is>
           <t>900 Ridge Rd</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
+      <c r="I10" t="inlineStr">
         <is>
           <t>Building C</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
+      <c r="J10" t="inlineStr">
         <is>
           <t>Denver</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr">
+      <c r="K10" t="inlineStr">
         <is>
           <t>CO</t>
         </is>
       </c>
-      <c r="K10" s="10" t="inlineStr">
+      <c r="L10" s="10" t="inlineStr">
         <is>
           <t>80202</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr">
+      <c r="M10" t="inlineStr">
         <is>
           <t>USA</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr">
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>Billing</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
         <is>
           <t>303-555-0500</t>
         </is>
       </c>
-      <c r="O10" t="inlineStr">
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>Office</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>Support</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
         <is>
           <t>support@summitdata.example</t>
         </is>
       </c>
-      <c r="P10" t="inlineStr">
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>24/7 support</t>
+        </is>
+      </c>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>eng</t>
+        </is>
+      </c>
+      <c r="X10" t="inlineStr">
+        <is>
+          <t>Support</t>
+        </is>
+      </c>
+      <c r="Y10" t="inlineStr">
         <is>
           <t>https://www.summitdata.example</t>
         </is>
       </c>
-      <c r="T10" t="inlineStr">
+      <c r="AD10" t="inlineStr">
         <is>
           <t>Access Provider</t>
         </is>
@@ -2357,42 +2532,42 @@
           <t>Cedar Archive Foundation</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="E11" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="F11" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="G11" t="inlineStr">
         <is>
           <t>Nonprofit foundation supporting regional archives.</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
+      <c r="H11" t="inlineStr">
         <is>
           <t>4 Cedar Ct</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr">
+      <c r="J11" t="inlineStr">
         <is>
           <t>Portland</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr">
+      <c r="K11" t="inlineStr">
         <is>
           <t>OR</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr">
+      <c r="L11" t="inlineStr">
         <is>
           <t>97201</t>
         </is>
       </c>
-      <c r="L11" t="inlineStr">
+      <c r="M11" t="inlineStr">
         <is>
           <t>USA</t>
         </is>
@@ -2409,57 +2584,62 @@
           <t>Lone Star Publishing</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="E12" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="F12" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="G12" t="inlineStr">
         <is>
           <t>Regional publisher of Texas history titles.</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr">
+      <c r="H12" t="inlineStr">
         <is>
           <t>210 Alamo St</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr">
+      <c r="J12" t="inlineStr">
         <is>
           <t>San Antonio</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr">
+      <c r="K12" t="inlineStr">
         <is>
           <t>TX</t>
         </is>
       </c>
-      <c r="K12" s="11" t="inlineStr">
+      <c r="L12" s="11" t="inlineStr">
         <is>
           <t>78205</t>
         </is>
       </c>
-      <c r="L12" t="inlineStr">
+      <c r="M12" t="inlineStr">
         <is>
           <t>USA</t>
         </is>
       </c>
-      <c r="M12" t="inlineStr">
+      <c r="P12" t="inlineStr">
         <is>
           <t>210-555-0600</t>
         </is>
       </c>
-      <c r="O12" s="7" t="inlineStr">
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>Office</t>
+        </is>
+      </c>
+      <c r="U12" s="7" t="inlineStr">
         <is>
           <t>orders@lonestarpub.example</t>
         </is>
       </c>
-      <c r="T12" t="inlineStr">
+      <c r="AD12" t="inlineStr">
         <is>
           <t>Publisher</t>
         </is>
@@ -2481,18 +2661,18 @@
           <t>MV Consortium</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="E13" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="F13" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="O13" s="7" t="n"/>
-      <c r="P13" s="7" t="n"/>
+      <c r="U13" s="7" t="n"/>
+      <c r="Y13" s="7" t="n"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2505,62 +2685,77 @@
           <t>Blue Horizon Media</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="E14" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="F14" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="G14" t="inlineStr">
         <is>
           <t>Streaming and digital media licensing.</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
+      <c r="H14" t="inlineStr">
         <is>
           <t>88 Harbor Way</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr">
+      <c r="J14" t="inlineStr">
         <is>
           <t>Seattle</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr">
+      <c r="K14" t="inlineStr">
         <is>
           <t>WA</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr">
+      <c r="L14" t="inlineStr">
         <is>
           <t>98101</t>
         </is>
       </c>
-      <c r="L14" t="inlineStr">
+      <c r="M14" t="inlineStr">
         <is>
           <t>USA</t>
         </is>
       </c>
-      <c r="M14" t="inlineStr">
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>Licensing</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
         <is>
           <t>206-555-0700</t>
         </is>
       </c>
-      <c r="O14" s="7" t="inlineStr">
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>Office</t>
+        </is>
+      </c>
+      <c r="U14" s="7" t="inlineStr">
         <is>
           <t>licensing@bluehorizon.example</t>
         </is>
       </c>
-      <c r="P14" s="7" t="inlineStr">
+      <c r="X14" t="inlineStr">
+        <is>
+          <t>Licensing</t>
+        </is>
+      </c>
+      <c r="Y14" s="7" t="inlineStr">
         <is>
           <t>https://www.bluehorizon.example</t>
         </is>
       </c>
-      <c r="T14" t="inlineStr">
+      <c r="AD14" t="inlineStr">
         <is>
           <t>Content Provider</t>
         </is>
@@ -2577,17 +2772,17 @@
           <t>Greenfield Historical Society</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="E15" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="F15" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
+      <c r="G15" t="inlineStr">
         <is>
           <t>Local historical society; donor of archival materials.</t>
         </is>
@@ -2604,34 +2799,39 @@
           <t>Red Rock Bindery</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="E16" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="F16" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
+      <c r="G16" t="inlineStr">
         <is>
           <t>Book binding and repair services.</t>
         </is>
       </c>
-      <c r="K16" s="10" t="n"/>
-      <c r="M16" t="inlineStr">
+      <c r="L16" s="10" t="n"/>
+      <c r="P16" t="inlineStr">
         <is>
           <t>480-555-0800</t>
         </is>
       </c>
-      <c r="O16" s="7" t="inlineStr">
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>Office</t>
+        </is>
+      </c>
+      <c r="U16" s="7" t="inlineStr">
         <is>
           <t>service@redrockbind.example</t>
         </is>
       </c>
-      <c r="P16" s="7" t="n"/>
-      <c r="T16" t="inlineStr">
+      <c r="Y16" s="7" t="n"/>
+      <c r="AD16" t="inlineStr">
         <is>
           <t>Material Supplier</t>
         </is>
@@ -2648,52 +2848,57 @@
           <t>Silverlake Digital</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="E17" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="F17" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
+      <c r="G17" t="inlineStr">
         <is>
           <t>Digital repository hosting.</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr">
+      <c r="H17" t="inlineStr">
         <is>
           <t>15 Lakeview Dr</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr">
+      <c r="J17" t="inlineStr">
         <is>
           <t>Madison</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr">
+      <c r="K17" t="inlineStr">
         <is>
           <t>WI</t>
         </is>
       </c>
-      <c r="K17" t="inlineStr">
+      <c r="L17" t="inlineStr">
         <is>
           <t>53703</t>
         </is>
       </c>
-      <c r="L17" t="inlineStr">
+      <c r="M17" t="inlineStr">
         <is>
           <t>USA</t>
         </is>
       </c>
-      <c r="O17" s="7" t="inlineStr">
+      <c r="U17" s="7" t="inlineStr">
         <is>
           <t>support@silverlake.example</t>
         </is>
       </c>
-      <c r="T17" t="inlineStr">
+      <c r="X17" t="inlineStr">
+        <is>
+          <t>Support</t>
+        </is>
+      </c>
+      <c r="AD17" t="inlineStr">
         <is>
           <t>Access Provider</t>
         </is>
@@ -2710,54 +2915,64 @@
           <t>Amberwave Distribution</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="E18" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
+      <c r="F18" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
+      <c r="G18" t="inlineStr">
         <is>
           <t>Wholesale distributor of periodicals.</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr">
+      <c r="H18" t="inlineStr">
         <is>
           <t>300 Commerce Pkwy</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr">
+      <c r="J18" t="inlineStr">
         <is>
           <t>Columbus</t>
         </is>
       </c>
-      <c r="J18" t="inlineStr">
+      <c r="K18" t="inlineStr">
         <is>
           <t>OH</t>
         </is>
       </c>
-      <c r="K18" t="inlineStr">
+      <c r="L18" t="inlineStr">
         <is>
           <t>43215</t>
         </is>
       </c>
-      <c r="L18" t="inlineStr">
+      <c r="M18" t="inlineStr">
         <is>
           <t>USA</t>
         </is>
       </c>
-      <c r="M18" t="inlineStr">
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>Shipping</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
         <is>
           <t>614-555-0900</t>
         </is>
       </c>
-      <c r="O18" s="7" t="n"/>
-      <c r="P18" s="7" t="n"/>
-      <c r="T18" t="inlineStr">
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>Office</t>
+        </is>
+      </c>
+      <c r="U18" s="7" t="n"/>
+      <c r="Y18" s="7" t="n"/>
+      <c r="AD18" t="inlineStr">
         <is>
           <t>Vendor</t>
         </is>
@@ -2774,22 +2989,22 @@
           <t>Iron Gate Records Management</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="E19" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
+      <c r="F19" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
+      <c r="G19" t="inlineStr">
         <is>
           <t>Off-site records storage.</t>
         </is>
       </c>
-      <c r="M19" s="12" t="n"/>
+      <c r="P19" s="12" t="n"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2802,23 +3017,23 @@
           <t>Crystal Springs Friends Group</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="E20" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
+      <c r="F20" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
+      <c r="G20" t="inlineStr">
         <is>
           <t>Volunteer group supporting the Crystal Springs branch library.</t>
         </is>
       </c>
-      <c r="O20" s="7" t="n"/>
-      <c r="P20" s="7" t="n"/>
+      <c r="U20" s="7" t="n"/>
+      <c r="Y20" s="7" t="n"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2831,57 +3046,62 @@
           <t>Timberline Learning Resources</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="E21" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
+      <c r="F21" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr">
+      <c r="G21" t="inlineStr">
         <is>
           <t>K-12 and academic learning resource vendor.</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr">
+      <c r="H21" t="inlineStr">
         <is>
           <t>42 Ridgeline Rd</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr">
+      <c r="J21" t="inlineStr">
         <is>
           <t>Boise</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr">
+      <c r="K21" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="K21" t="inlineStr">
+      <c r="L21" t="inlineStr">
         <is>
           <t>83702</t>
         </is>
       </c>
-      <c r="L21" t="inlineStr">
+      <c r="M21" t="inlineStr">
         <is>
           <t>USA</t>
         </is>
       </c>
-      <c r="O21" s="7" t="inlineStr">
+      <c r="U21" s="7" t="inlineStr">
         <is>
           <t>sales@timberline.example</t>
         </is>
       </c>
-      <c r="P21" s="7" t="inlineStr">
+      <c r="X21" t="inlineStr">
+        <is>
+          <t>Sales</t>
+        </is>
+      </c>
+      <c r="Y21" s="7" t="inlineStr">
         <is>
           <t>https://www.timberline.example</t>
         </is>
       </c>
-      <c r="T21" t="inlineStr">
+      <c r="AD21" t="inlineStr">
         <is>
           <t>Content Provider</t>
         </is>
@@ -2898,23 +3118,23 @@
           <t>Coastal Archives Cooperative</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="E22" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
+      <c r="F22" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr">
+      <c r="G22" t="inlineStr">
         <is>
           <t>Regional cooperative for shared archival storage.</t>
         </is>
       </c>
-      <c r="O22" s="7" t="n"/>
-      <c r="P22" s="7" t="n"/>
+      <c r="U22" s="7" t="n"/>
+      <c r="Y22" s="7" t="n"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2927,32 +3147,37 @@
           <t>Willow Data Services</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="E23" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
+      <c r="F23" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
+      <c r="G23" t="inlineStr">
         <is>
           <t>Metadata enrichment and data cleanup services.</t>
         </is>
       </c>
-      <c r="M23" t="inlineStr">
+      <c r="P23" t="inlineStr">
         <is>
           <t>651-555-1000</t>
         </is>
       </c>
-      <c r="O23" s="7" t="inlineStr">
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>Office</t>
+        </is>
+      </c>
+      <c r="U23" s="7" t="inlineStr">
         <is>
           <t>projects@willowdata.example</t>
         </is>
       </c>
-      <c r="T23" t="inlineStr">
+      <c r="AD23" t="inlineStr">
         <is>
           <t>Service Provider</t>
         </is>
@@ -2969,23 +3194,23 @@
           <t>Stonebridge Consortium</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="E24" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
+      <c r="F24" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr">
+      <c r="G24" t="inlineStr">
         <is>
           <t>Multi-library resource-sharing consortium.</t>
         </is>
       </c>
-      <c r="O24" s="7" t="n"/>
-      <c r="P24" s="7" t="n"/>
+      <c r="U24" s="7" t="n"/>
+      <c r="Y24" s="7" t="n"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2998,80 +3223,97 @@
           <t>Falcon Media Group</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="E25" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
+      <c r="F25" t="inlineStr">
         <is>
           <t>Inactive</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr">
+      <c r="G25" t="inlineStr">
         <is>
           <t>Media licensing vendor; contract not renewed.</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr">
+      <c r="H25" t="inlineStr">
         <is>
           <t>10 Falcon Ct</t>
         </is>
       </c>
-      <c r="I25" t="inlineStr">
+      <c r="J25" t="inlineStr">
         <is>
           <t>Phoenix</t>
         </is>
       </c>
-      <c r="J25" t="inlineStr">
+      <c r="K25" t="inlineStr">
         <is>
           <t>AZ</t>
         </is>
       </c>
-      <c r="K25" t="inlineStr">
+      <c r="L25" t="inlineStr">
         <is>
           <t>85001</t>
         </is>
       </c>
-      <c r="L25" t="inlineStr">
+      <c r="M25" t="inlineStr">
         <is>
           <t>USA</t>
         </is>
       </c>
-      <c r="M25" t="inlineStr">
+      <c r="P25" t="inlineStr">
         <is>
           <t>602-555-1100</t>
         </is>
       </c>
-      <c r="O25" s="7" t="n"/>
-      <c r="P25" s="7" t="n"/>
-      <c r="T25" t="inlineStr">
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>Office</t>
+        </is>
+      </c>
+      <c r="U25" s="7" t="n"/>
+      <c r="Y25" s="7" t="n"/>
+      <c r="AD25" t="inlineStr">
         <is>
           <t>Content Provider</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="O26" s="7" t="n"/>
-      <c r="P26" s="7" t="n"/>
+      <c r="U26" s="7" t="n"/>
+      <c r="Y26" s="7" t="n"/>
     </row>
     <row r="27">
-      <c r="O27" s="7" t="n"/>
-      <c r="P27" s="7" t="n"/>
+      <c r="U27" s="7" t="n"/>
+      <c r="Y27" s="7" t="n"/>
     </row>
     <row r="28">
-      <c r="P28" s="7" t="n"/>
+      <c r="Y28" s="7" t="n"/>
     </row>
   </sheetData>
-  <dataValidations count="3">
-    <dataValidation sqref="D6:D1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+  <dataValidations count="7">
+    <dataValidation sqref="E6:E1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes, No"</formula1>
     </dataValidation>
-    <dataValidation sqref="E6:E1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F6:F1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Active, Inactive, Pending"</formula1>
     </dataValidation>
-    <dataValidation sqref="T6:T1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="AD6:AD1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Access provider,Auction house,Book trade,Consortium,Content provider,Logistics,Material supplier,Membership organization,Private person,Publisher"</formula1>
+    </dataValidation>
+    <dataValidation sqref="O6:O1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Accounts Payable,Administrative,Claims and queries,Customer Service,Licensing,Payments,Receiving orders,Returns,Sales,Shipments,Support"</formula1>
+    </dataValidation>
+    <dataValidation sqref="Q6:Q1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Office, Mobile, Fax, Other"</formula1>
+    </dataValidation>
+    <dataValidation sqref="S6:S1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Accounts Payable,Administrative,Claims and queries,Customer Service,Licensing,Payments,Receiving orders,Returns,Sales,Shipments,Support"</formula1>
+    </dataValidation>
+    <dataValidation sqref="X6:X1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Accounts Payable,Administrative,Claims and queries,Customer Service,Licensing,Payments,Receiving orders,Returns,Sales,Shipments,Support"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3590,7 +3832,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:D7"/>
+  <dimension ref="A2:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18.140625" customWidth="1" style="23" min="1" max="1"/>
@@ -3618,6 +3860,11 @@
       </c>
       <c r="D2" s="32" t="inlineStr">
         <is>
+          <t>LANGUAGE</t>
+        </is>
+      </c>
+      <c r="E2" s="32" t="inlineStr">
+        <is>
           <t>CATEGORIES</t>
         </is>
       </c>
@@ -3662,7 +3909,7 @@
           <t>sales@northstarlib.example</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>Sales</t>
         </is>
@@ -3684,7 +3931,7 @@
           <t>Conservation team</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>Support</t>
         </is>
@@ -3704,7 +3951,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="D3:D1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E3:E1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Accounts Payable,Administrative,Claims and queries,Customer Service,Licensing,Payments,Receiving orders,Returns,Sales,Shipments,Support"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>